<commit_message>
commit final model params
</commit_message>
<xml_diff>
--- a/Y2A_model_iteration_log.xlsx
+++ b/Y2A_model_iteration_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koenm\Documents\repositorys\year_2\fae2-nlpr-group-group-4-1\fae2-nlpr-group-group-4-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC220CA-716D-4FAB-A816-689B479F9B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7606724-4C26-475A-BF44-40D67EF6222A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
@@ -1199,16 +1199,16 @@
         <v>33</v>
       </c>
       <c r="K11" s="10">
-        <v>0.38400000000000001</v>
+        <v>0.49399999999999999</v>
       </c>
       <c r="L11" s="10">
-        <v>0.5</v>
+        <v>0.54</v>
       </c>
       <c r="M11" s="10">
-        <v>0.38400000000000001</v>
+        <v>0.49399999999999999</v>
       </c>
       <c r="N11" s="10">
-        <v>0.38400000000000001</v>
+        <v>0.42599999999999999</v>
       </c>
       <c r="O11" s="10"/>
       <c r="P11" s="10" t="s">

</xml_diff>